<commit_message>
[NCBI Daily] 2026-09-01 pipeline results
</commit_message>
<xml_diff>
--- a/results/2026-09-01/NCBI_Eukaryota_Taxonomy_Summary.xlsx
+++ b/results/2026-09-01/NCBI_Eukaryota_Taxonomy_Summary.xlsx
@@ -469,7 +469,7 @@
         <v>42040</v>
       </c>
       <c r="F2" t="n">
-        <v>766662</v>
+        <v>766666</v>
       </c>
     </row>
     <row r="3">
@@ -490,10 +490,10 @@
         <v>482</v>
       </c>
       <c r="E3" t="n">
-        <v>14532</v>
+        <v>14531</v>
       </c>
       <c r="F3" t="n">
-        <v>334994</v>
+        <v>336685</v>
       </c>
     </row>
     <row r="4">
@@ -514,10 +514,10 @@
         <v>647</v>
       </c>
       <c r="E4" t="n">
-        <v>5337</v>
+        <v>5340</v>
       </c>
       <c r="F4" t="n">
-        <v>77484</v>
+        <v>77497</v>
       </c>
     </row>
     <row r="5">
@@ -541,7 +541,7 @@
         <v>1641</v>
       </c>
       <c r="F5" t="n">
-        <v>56541</v>
+        <v>56553</v>
       </c>
     </row>
     <row r="6">
@@ -562,10 +562,10 @@
         <v>559</v>
       </c>
       <c r="E6" t="n">
-        <v>4797</v>
+        <v>4798</v>
       </c>
       <c r="F6" t="n">
-        <v>52815</v>
+        <v>52818</v>
       </c>
     </row>
     <row r="7">
@@ -589,7 +589,7 @@
         <v>1749</v>
       </c>
       <c r="F7" t="n">
-        <v>41776</v>
+        <v>41780</v>
       </c>
     </row>
     <row r="8">
@@ -637,7 +637,7 @@
         <v>4083</v>
       </c>
       <c r="F9" t="n">
-        <v>32086</v>
+        <v>32088</v>
       </c>
     </row>
     <row r="10">
@@ -709,7 +709,7 @@
         <v>623</v>
       </c>
       <c r="F12" t="n">
-        <v>14656</v>
+        <v>14657</v>
       </c>
     </row>
     <row r="13">
@@ -733,7 +733,7 @@
         <v>1218</v>
       </c>
       <c r="F13" t="n">
-        <v>14581</v>
+        <v>14582</v>
       </c>
     </row>
     <row r="14">
@@ -781,7 +781,7 @@
         <v>904</v>
       </c>
       <c r="F15" t="n">
-        <v>11836</v>
+        <v>11841</v>
       </c>
     </row>
     <row r="16">
@@ -826,10 +826,10 @@
         <v>86</v>
       </c>
       <c r="E17" t="n">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="F17" t="n">
-        <v>11731</v>
+        <v>11733</v>
       </c>
     </row>
     <row r="18">
@@ -853,7 +853,7 @@
         <v>2438</v>
       </c>
       <c r="F18" t="n">
-        <v>11284</v>
+        <v>11285</v>
       </c>
     </row>
     <row r="19">
@@ -901,7 +901,7 @@
         <v>1440</v>
       </c>
       <c r="F20" t="n">
-        <v>10186</v>
+        <v>10195</v>
       </c>
     </row>
     <row r="21">
@@ -925,7 +925,7 @@
         <v>877</v>
       </c>
       <c r="F21" t="n">
-        <v>9763</v>
+        <v>9762</v>
       </c>
     </row>
     <row r="22">
@@ -1405,7 +1405,7 @@
         <v>523</v>
       </c>
       <c r="F41" t="n">
-        <v>2855</v>
+        <v>2856</v>
       </c>
     </row>
     <row r="42">
@@ -1477,7 +1477,7 @@
         <v>416</v>
       </c>
       <c r="F44" t="n">
-        <v>2739</v>
+        <v>2740</v>
       </c>
     </row>
     <row r="45">
@@ -1501,7 +1501,7 @@
         <v>90</v>
       </c>
       <c r="F45" t="n">
-        <v>2729</v>
+        <v>2730</v>
       </c>
     </row>
     <row r="46">
@@ -1957,7 +1957,7 @@
         <v>188</v>
       </c>
       <c r="F64" t="n">
-        <v>1342</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="65">
@@ -2125,7 +2125,7 @@
         <v>267</v>
       </c>
       <c r="F71" t="n">
-        <v>1243</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="72">
@@ -2221,7 +2221,7 @@
         <v>90</v>
       </c>
       <c r="F75" t="n">
-        <v>1131</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="76">
@@ -2635,49 +2635,49 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Oomycota</t>
+          <t>Parabasalia</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Saprolegniomycetes</t>
+          <t>unclassified Parabasalia class</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D93" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="E93" t="n">
-        <v>36</v>
+        <v>91</v>
       </c>
       <c r="F93" t="n">
-        <v>652</v>
+        <v>656</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Parabasalia</t>
+          <t>Oomycota</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>unclassified Parabasalia class</t>
+          <t>Saprolegniomycetes</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="D94" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>91</v>
+        <v>36</v>
       </c>
       <c r="F94" t="n">
-        <v>649</v>
+        <v>652</v>
       </c>
     </row>
     <row r="95">
@@ -3229,7 +3229,7 @@
         <v>44</v>
       </c>
       <c r="F117" t="n">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="118">
@@ -3931,46 +3931,46 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Streptophyta</t>
+          <t>Preaxostyla</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Anthocerotopsida</t>
+          <t>unclassified Preaxostyla class</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D147" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E147" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F147" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Preaxostyla</t>
+          <t>Streptophyta</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>unclassified Preaxostyla class</t>
+          <t>Anthocerotopsida</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D148" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E148" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F148" t="n">
         <v>199</v>
@@ -7147,22 +7147,22 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Ciliophora</t>
+          <t>unclassified cellular organisms phylum</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Odontostomatea</t>
+          <t>Jakobea</t>
         </is>
       </c>
       <c r="C281" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D281" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E281" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F281" t="n">
         <v>20</v>
@@ -7171,36 +7171,36 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Chlorophyta</t>
+          <t>Ciliophora</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Chloropicophyceae</t>
+          <t>Odontostomatea</t>
         </is>
       </c>
       <c r="C282" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D282" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E282" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F282" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Ascomycota</t>
+          <t>Chlorophyta</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Sareomycetes</t>
+          <t>Chloropicophyceae</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -7210,7 +7210,7 @@
         <v>2</v>
       </c>
       <c r="E283" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F283" t="n">
         <v>19</v>
@@ -7219,22 +7219,22 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>unclassified Metazoa phylum</t>
+          <t>Ascomycota</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>unclassified Metazoa class</t>
+          <t>Sareomycetes</t>
         </is>
       </c>
       <c r="C284" t="n">
         <v>1</v>
       </c>
       <c r="D284" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E284" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F284" t="n">
         <v>19</v>
@@ -7243,22 +7243,22 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Tubulinea</t>
+          <t>unclassified Metazoa phylum</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Echinamoebida</t>
+          <t>unclassified Metazoa class</t>
         </is>
       </c>
       <c r="C285" t="n">
         <v>1</v>
       </c>
       <c r="D285" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E285" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F285" t="n">
         <v>19</v>
@@ -7267,22 +7267,22 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>unclassified cellular organisms phylum</t>
+          <t>Tubulinea</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Jakobea</t>
+          <t>Echinamoebida</t>
         </is>
       </c>
       <c r="C286" t="n">
         <v>1</v>
       </c>
       <c r="D286" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E286" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F286" t="n">
         <v>19</v>

</xml_diff>